<commit_message>
correcion de nombres de integrantes
</commit_message>
<xml_diff>
--- a/Fase 1/Evidencias Grupales/PLANILLA DE EVALUACIÓN FASE 1.xlsx
+++ b/Fase 1/Evidencias Grupales/PLANILLA DE EVALUACIÓN FASE 1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CETECOM\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Capstone\Fase 1\Evidencias Grupales\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AE6866CD-F43D-4709-9EEB-5232FDFF29D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18590069-41CF-41F0-B542-ADB41AE7F936}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EVALUACION1" sheetId="1" r:id="rId1"/>
@@ -59,15 +59,12 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="98">
   <si>
     <t>INTEGRANTES</t>
   </si>
@@ -381,10 +378,13 @@
     <t>Muy Relevante</t>
   </si>
   <si>
-    <t>SANCHEZ CARIS VICENTE ANDRES</t>
+    <t>MOISES MARINO SANCHEZ LINARES</t>
   </si>
   <si>
-    <t>COILLA NUÑEZ DENISSE MARION</t>
+    <t>DENISSE MARION COILLA NUNEZ</t>
+  </si>
+  <si>
+    <t>NAYERLY DEL CARMEN YANEZ GATICA</t>
   </si>
 </sst>
 </file>
@@ -1050,34 +1050,34 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="255"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="255"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
@@ -1114,7 +1114,7 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1150,9 +1150,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1190,7 +1190,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1296,7 +1296,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1438,7 +1438,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1531,7 +1531,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="32" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C6" s="6">
         <f>EVALUACION1!$C$24</f>
@@ -1552,22 +1552,22 @@
         <v>3</v>
       </c>
       <c r="B11" s="14"/>
-      <c r="C11" s="51" t="s">
+      <c r="C11" s="57" t="s">
         <v>4</v>
       </c>
       <c r="D11" s="58" t="s">
         <v>5</v>
       </c>
-      <c r="E11" s="62"/>
-      <c r="F11" s="62"/>
-      <c r="G11" s="62"/>
-      <c r="H11" s="62"/>
-      <c r="I11" s="62"/>
-      <c r="J11" s="62"/>
-      <c r="K11" s="59"/>
+      <c r="E11" s="59"/>
+      <c r="F11" s="59"/>
+      <c r="G11" s="59"/>
+      <c r="H11" s="59"/>
+      <c r="I11" s="59"/>
+      <c r="J11" s="59"/>
+      <c r="K11" s="60"/>
     </row>
     <row r="12" spans="1:11" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="61"/>
+      <c r="A12" s="62"/>
       <c r="B12" s="24" t="s">
         <v>6</v>
       </c>
@@ -1575,19 +1575,19 @@
       <c r="D12" s="58" t="s">
         <v>7</v>
       </c>
-      <c r="E12" s="59"/>
+      <c r="E12" s="60"/>
       <c r="F12" s="58" t="s">
         <v>8</v>
       </c>
-      <c r="G12" s="59"/>
+      <c r="G12" s="60"/>
       <c r="H12" s="58" t="s">
         <v>9</v>
       </c>
-      <c r="I12" s="59"/>
+      <c r="I12" s="60"/>
       <c r="J12" s="58" t="s">
         <v>10</v>
       </c>
-      <c r="K12" s="59"/>
+      <c r="K12" s="60"/>
     </row>
     <row r="13" spans="1:11" ht="24" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A13" s="65"/>
@@ -2011,7 +2011,7 @@
       </c>
     </row>
     <row r="23" spans="1:11" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="61"/>
+      <c r="A23" s="62"/>
       <c r="B23" s="34" t="s">
         <v>11</v>
       </c>
@@ -2053,59 +2053,59 @@
     <row r="25" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="26" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="27" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="60" t="s">
+      <c r="A27" s="61" t="s">
         <v>13</v>
       </c>
       <c r="B27" s="49" t="s">
         <v>14</v>
       </c>
-      <c r="C27" s="52" t="str">
+      <c r="C27" s="51" t="str">
         <f>$B$4</f>
-        <v>SANCHEZ CARIS VICENTE ANDRES</v>
-      </c>
-      <c r="D27" s="53"/>
-      <c r="E27" s="53"/>
-      <c r="F27" s="53"/>
-      <c r="G27" s="53"/>
-      <c r="H27" s="53"/>
-      <c r="I27" s="53"/>
-      <c r="J27" s="53"/>
-      <c r="K27" s="54"/>
+        <v>MOISES MARINO SANCHEZ LINARES</v>
+      </c>
+      <c r="D27" s="52"/>
+      <c r="E27" s="52"/>
+      <c r="F27" s="52"/>
+      <c r="G27" s="52"/>
+      <c r="H27" s="52"/>
+      <c r="I27" s="52"/>
+      <c r="J27" s="52"/>
+      <c r="K27" s="53"/>
     </row>
     <row r="28" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="61"/>
+      <c r="A28" s="62"/>
       <c r="B28" s="50"/>
-      <c r="C28" s="55"/>
-      <c r="D28" s="56"/>
-      <c r="E28" s="56"/>
-      <c r="F28" s="56"/>
-      <c r="G28" s="56"/>
-      <c r="H28" s="56"/>
-      <c r="I28" s="56"/>
-      <c r="J28" s="56"/>
-      <c r="K28" s="57"/>
+      <c r="C28" s="54"/>
+      <c r="D28" s="55"/>
+      <c r="E28" s="55"/>
+      <c r="F28" s="55"/>
+      <c r="G28" s="55"/>
+      <c r="H28" s="55"/>
+      <c r="I28" s="55"/>
+      <c r="J28" s="55"/>
+      <c r="K28" s="56"/>
     </row>
     <row r="29" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="61"/>
+      <c r="A29" s="62"/>
       <c r="B29" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C29" s="51" t="s">
+      <c r="C29" s="57" t="s">
         <v>4</v>
       </c>
       <c r="D29" s="58" t="s">
         <v>5</v>
       </c>
-      <c r="E29" s="62"/>
-      <c r="F29" s="62"/>
-      <c r="G29" s="62"/>
-      <c r="H29" s="62"/>
-      <c r="I29" s="62"/>
-      <c r="J29" s="62"/>
-      <c r="K29" s="59"/>
+      <c r="E29" s="59"/>
+      <c r="F29" s="59"/>
+      <c r="G29" s="59"/>
+      <c r="H29" s="59"/>
+      <c r="I29" s="59"/>
+      <c r="J29" s="59"/>
+      <c r="K29" s="60"/>
     </row>
     <row r="30" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="61"/>
+      <c r="A30" s="62"/>
       <c r="B30" s="15" t="s">
         <v>6</v>
       </c>
@@ -2113,22 +2113,22 @@
       <c r="D30" s="58" t="s">
         <v>7</v>
       </c>
-      <c r="E30" s="59"/>
+      <c r="E30" s="60"/>
       <c r="F30" s="58" t="s">
         <v>8</v>
       </c>
-      <c r="G30" s="59"/>
+      <c r="G30" s="60"/>
       <c r="H30" s="58" t="s">
         <v>16</v>
       </c>
-      <c r="I30" s="59"/>
+      <c r="I30" s="60"/>
       <c r="J30" s="58" t="s">
         <v>10</v>
       </c>
-      <c r="K30" s="59"/>
+      <c r="K30" s="60"/>
     </row>
     <row r="31" spans="1:11" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="61"/>
+      <c r="A31" s="62"/>
       <c r="B31" s="35" t="str">
         <f>RUBRICA!A7</f>
         <v>3. Relaciona el Proyecto APT con sus intereses profesionales. *</v>
@@ -2170,7 +2170,7 @@
       </c>
     </row>
     <row r="32" spans="1:11" ht="25.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="61"/>
+      <c r="A32" s="62"/>
       <c r="B32" s="35" t="str">
         <f>RUBRICA!A15</f>
         <v>11. Expone el tema utilizando un lenguaje técnico disciplinar al presentar la propuesta y responde evidenciando un manejo de la información. *</v>
@@ -2212,7 +2212,7 @@
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A33" s="61"/>
+      <c r="A33" s="62"/>
       <c r="B33" s="35" t="str">
         <f>RUBRICA!A17</f>
         <v>13. Colaboración y trabajo en equipo *</v>
@@ -2254,7 +2254,7 @@
       </c>
     </row>
     <row r="34" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="61"/>
+      <c r="A34" s="62"/>
       <c r="B34" s="21" t="s">
         <v>17</v>
       </c>
@@ -2303,59 +2303,59 @@
     </row>
     <row r="38" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="39" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="60" t="s">
+      <c r="A39" s="61" t="s">
         <v>13</v>
       </c>
       <c r="B39" s="49" t="s">
         <v>14</v>
       </c>
-      <c r="C39" s="52" t="str">
+      <c r="C39" s="51" t="str">
         <f>B5</f>
-        <v>COILLA NUÑEZ DENISSE MARION</v>
-      </c>
-      <c r="D39" s="53"/>
-      <c r="E39" s="53"/>
-      <c r="F39" s="53"/>
-      <c r="G39" s="53"/>
-      <c r="H39" s="53"/>
-      <c r="I39" s="53"/>
-      <c r="J39" s="53"/>
-      <c r="K39" s="54"/>
+        <v>DENISSE MARION COILLA NUNEZ</v>
+      </c>
+      <c r="D39" s="52"/>
+      <c r="E39" s="52"/>
+      <c r="F39" s="52"/>
+      <c r="G39" s="52"/>
+      <c r="H39" s="52"/>
+      <c r="I39" s="52"/>
+      <c r="J39" s="52"/>
+      <c r="K39" s="53"/>
     </row>
     <row r="40" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="61"/>
+      <c r="A40" s="62"/>
       <c r="B40" s="50"/>
-      <c r="C40" s="55"/>
-      <c r="D40" s="56"/>
-      <c r="E40" s="56"/>
-      <c r="F40" s="56"/>
-      <c r="G40" s="56"/>
-      <c r="H40" s="56"/>
-      <c r="I40" s="56"/>
-      <c r="J40" s="56"/>
-      <c r="K40" s="57"/>
+      <c r="C40" s="54"/>
+      <c r="D40" s="55"/>
+      <c r="E40" s="55"/>
+      <c r="F40" s="55"/>
+      <c r="G40" s="55"/>
+      <c r="H40" s="55"/>
+      <c r="I40" s="55"/>
+      <c r="J40" s="55"/>
+      <c r="K40" s="56"/>
     </row>
     <row r="41" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="61"/>
+      <c r="A41" s="62"/>
       <c r="B41" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C41" s="51" t="s">
+      <c r="C41" s="57" t="s">
         <v>4</v>
       </c>
       <c r="D41" s="58" t="s">
         <v>5</v>
       </c>
-      <c r="E41" s="62"/>
-      <c r="F41" s="62"/>
-      <c r="G41" s="62"/>
-      <c r="H41" s="62"/>
-      <c r="I41" s="62"/>
-      <c r="J41" s="62"/>
-      <c r="K41" s="59"/>
+      <c r="E41" s="59"/>
+      <c r="F41" s="59"/>
+      <c r="G41" s="59"/>
+      <c r="H41" s="59"/>
+      <c r="I41" s="59"/>
+      <c r="J41" s="59"/>
+      <c r="K41" s="60"/>
     </row>
     <row r="42" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="61"/>
+      <c r="A42" s="62"/>
       <c r="B42" s="15" t="s">
         <v>6</v>
       </c>
@@ -2363,22 +2363,22 @@
       <c r="D42" s="58" t="s">
         <v>7</v>
       </c>
-      <c r="E42" s="59"/>
+      <c r="E42" s="60"/>
       <c r="F42" s="58" t="s">
         <v>8</v>
       </c>
-      <c r="G42" s="59"/>
+      <c r="G42" s="60"/>
       <c r="H42" s="58" t="s">
         <v>16</v>
       </c>
-      <c r="I42" s="59"/>
+      <c r="I42" s="60"/>
       <c r="J42" s="58" t="s">
         <v>10</v>
       </c>
-      <c r="K42" s="59"/>
+      <c r="K42" s="60"/>
     </row>
     <row r="43" spans="1:11" ht="25.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="61"/>
+      <c r="A43" s="62"/>
       <c r="B43" s="35" t="str">
         <f>RUBRICA!A7</f>
         <v>3. Relaciona el Proyecto APT con sus intereses profesionales. *</v>
@@ -2420,7 +2420,7 @@
       </c>
     </row>
     <row r="44" spans="1:11" ht="24" x14ac:dyDescent="0.25">
-      <c r="A44" s="61"/>
+      <c r="A44" s="62"/>
       <c r="B44" s="35" t="str">
         <f>RUBRICA!A15</f>
         <v>11. Expone el tema utilizando un lenguaje técnico disciplinar al presentar la propuesta y responde evidenciando un manejo de la información. *</v>
@@ -2462,7 +2462,7 @@
       </c>
     </row>
     <row r="45" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="61"/>
+      <c r="A45" s="62"/>
       <c r="B45" s="35" t="str">
         <f>RUBRICA!A17</f>
         <v>13. Colaboración y trabajo en equipo *</v>
@@ -2504,7 +2504,7 @@
       </c>
     </row>
     <row r="46" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="61"/>
+      <c r="A46" s="62"/>
       <c r="B46" s="21" t="s">
         <v>17</v>
       </c>
@@ -2552,59 +2552,59 @@
       <c r="C49" s="23"/>
     </row>
     <row r="50" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="60" t="s">
+      <c r="A50" s="61" t="s">
         <v>13</v>
       </c>
       <c r="B50" s="49" t="s">
         <v>14</v>
       </c>
-      <c r="C50" s="52" t="str">
+      <c r="C50" s="51" t="str">
         <f>B6</f>
-        <v>COILLA NUÑEZ DENISSE MARION</v>
-      </c>
-      <c r="D50" s="53"/>
-      <c r="E50" s="53"/>
-      <c r="F50" s="53"/>
-      <c r="G50" s="53"/>
-      <c r="H50" s="53"/>
-      <c r="I50" s="53"/>
-      <c r="J50" s="53"/>
-      <c r="K50" s="54"/>
+        <v>NAYERLY DEL CARMEN YANEZ GATICA</v>
+      </c>
+      <c r="D50" s="52"/>
+      <c r="E50" s="52"/>
+      <c r="F50" s="52"/>
+      <c r="G50" s="52"/>
+      <c r="H50" s="52"/>
+      <c r="I50" s="52"/>
+      <c r="J50" s="52"/>
+      <c r="K50" s="53"/>
     </row>
     <row r="51" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="61"/>
+      <c r="A51" s="62"/>
       <c r="B51" s="50"/>
-      <c r="C51" s="55"/>
-      <c r="D51" s="56"/>
-      <c r="E51" s="56"/>
-      <c r="F51" s="56"/>
-      <c r="G51" s="56"/>
-      <c r="H51" s="56"/>
-      <c r="I51" s="56"/>
-      <c r="J51" s="56"/>
-      <c r="K51" s="57"/>
+      <c r="C51" s="54"/>
+      <c r="D51" s="55"/>
+      <c r="E51" s="55"/>
+      <c r="F51" s="55"/>
+      <c r="G51" s="55"/>
+      <c r="H51" s="55"/>
+      <c r="I51" s="55"/>
+      <c r="J51" s="55"/>
+      <c r="K51" s="56"/>
     </row>
     <row r="52" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="61"/>
+      <c r="A52" s="62"/>
       <c r="B52" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C52" s="51" t="s">
+      <c r="C52" s="57" t="s">
         <v>4</v>
       </c>
       <c r="D52" s="58" t="s">
         <v>5</v>
       </c>
-      <c r="E52" s="62"/>
-      <c r="F52" s="62"/>
-      <c r="G52" s="62"/>
-      <c r="H52" s="62"/>
-      <c r="I52" s="62"/>
-      <c r="J52" s="62"/>
-      <c r="K52" s="59"/>
+      <c r="E52" s="59"/>
+      <c r="F52" s="59"/>
+      <c r="G52" s="59"/>
+      <c r="H52" s="59"/>
+      <c r="I52" s="59"/>
+      <c r="J52" s="59"/>
+      <c r="K52" s="60"/>
     </row>
     <row r="53" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="61"/>
+      <c r="A53" s="62"/>
       <c r="B53" s="15" t="s">
         <v>6</v>
       </c>
@@ -2612,22 +2612,22 @@
       <c r="D53" s="58" t="s">
         <v>7</v>
       </c>
-      <c r="E53" s="59"/>
+      <c r="E53" s="60"/>
       <c r="F53" s="58" t="s">
         <v>8</v>
       </c>
-      <c r="G53" s="59"/>
+      <c r="G53" s="60"/>
       <c r="H53" s="58" t="s">
         <v>16</v>
       </c>
-      <c r="I53" s="59"/>
+      <c r="I53" s="60"/>
       <c r="J53" s="58" t="s">
         <v>10</v>
       </c>
-      <c r="K53" s="59"/>
+      <c r="K53" s="60"/>
     </row>
     <row r="54" spans="1:11" ht="25.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="61"/>
+      <c r="A54" s="62"/>
       <c r="B54" s="35" t="str">
         <f>RUBRICA!A7</f>
         <v>3. Relaciona el Proyecto APT con sus intereses profesionales. *</v>
@@ -2669,7 +2669,7 @@
       </c>
     </row>
     <row r="55" spans="1:11" ht="24" x14ac:dyDescent="0.25">
-      <c r="A55" s="61"/>
+      <c r="A55" s="62"/>
       <c r="B55" s="35" t="str">
         <f>RUBRICA!A15</f>
         <v>11. Expone el tema utilizando un lenguaje técnico disciplinar al presentar la propuesta y responde evidenciando un manejo de la información. *</v>
@@ -2711,7 +2711,7 @@
       </c>
     </row>
     <row r="56" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="61"/>
+      <c r="A56" s="62"/>
       <c r="B56" s="35" t="str">
         <f>RUBRICA!A17</f>
         <v>13. Colaboración y trabajo en equipo *</v>
@@ -2753,7 +2753,7 @@
       </c>
     </row>
     <row r="57" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="61"/>
+      <c r="A57" s="62"/>
       <c r="B57" s="21" t="s">
         <v>17</v>
       </c>
@@ -3680,14 +3680,17 @@
     <row r="929" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="35">
-    <mergeCell ref="B39:B40"/>
-    <mergeCell ref="C39:K40"/>
-    <mergeCell ref="C41:C42"/>
-    <mergeCell ref="D41:K41"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="F42:G42"/>
-    <mergeCell ref="H42:I42"/>
-    <mergeCell ref="J42:K42"/>
+    <mergeCell ref="B50:B51"/>
+    <mergeCell ref="C52:C53"/>
+    <mergeCell ref="C50:K51"/>
+    <mergeCell ref="J53:K53"/>
+    <mergeCell ref="A50:A58"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="D52:K52"/>
+    <mergeCell ref="D53:E53"/>
+    <mergeCell ref="F53:G53"/>
+    <mergeCell ref="H53:I53"/>
     <mergeCell ref="A39:A47"/>
     <mergeCell ref="A27:A35"/>
     <mergeCell ref="E2:E3"/>
@@ -3704,17 +3707,14 @@
     <mergeCell ref="D29:K29"/>
     <mergeCell ref="D30:E30"/>
     <mergeCell ref="F30:G30"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="J30:K30"/>
-    <mergeCell ref="D52:K52"/>
-    <mergeCell ref="D53:E53"/>
-    <mergeCell ref="F53:G53"/>
-    <mergeCell ref="H53:I53"/>
-    <mergeCell ref="B50:B51"/>
-    <mergeCell ref="C52:C53"/>
-    <mergeCell ref="C50:K51"/>
-    <mergeCell ref="J53:K53"/>
-    <mergeCell ref="A50:A58"/>
+    <mergeCell ref="B39:B40"/>
+    <mergeCell ref="C39:K40"/>
+    <mergeCell ref="C41:C42"/>
+    <mergeCell ref="D41:K41"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="F42:G42"/>
+    <mergeCell ref="H42:I42"/>
+    <mergeCell ref="J42:K42"/>
   </mergeCells>
   <conditionalFormatting sqref="C4:E6">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="lessThan">

</xml_diff>